<commit_message>
feat: implement learning flow, Claude feedback, and Supabase integration
</commit_message>
<xml_diff>
--- a/curriculum-design/小論文添削サービス_カリキュラム設計.xlsx
+++ b/curriculum-design/小論文添削サービス_カリキュラム設計.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="R71ec54ac80944c08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_学習ロードマップ" sheetId="2" r:id="Rd874a38625994d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_段階別ルーブリック" sheetId="3" r:id="Rd450677042d449c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_日本語文成立チェック" sheetId="4" r:id="R1d4e3eeb8c2c4839"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_AI指示設計" sheetId="5" r:id="R761b033f401c46d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_API入出力契約" sheetId="6" r:id="Rae8f4315efda4b33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="R14e4c160643b4271"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_学習ロードマップ" sheetId="2" r:id="Red8171375d61473d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_段階別ルーブリック" sheetId="3" r:id="Rfcfa66b6cdc74f86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_日本語文成立チェック" sheetId="4" r:id="R7f3d7d52f2fd4089"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_AI指示設計" sheetId="5" r:id="R4ace695212de4193"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_API入出力契約" sheetId="6" r:id="Rbd01883ed37740d2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -527,7 +527,7 @@
   <x:dxfs count="3">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEBF7"/>
         </x:patternFill>
       </x:fill>
@@ -537,14 +537,14 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1006,13 +1006,13 @@
         <x:v>一文を成立させる</x:v>
       </x:c>
       <x:c r="D5" s="46" t="str">
-        <x:v>主語と述語が対応する一文を書く</x:v>
+        <x:v>「誰が・何が」と「どうする・どのようだ」を入れ、最後まで一文を書く</x:v>
       </x:c>
       <x:c r="E5" s="46" t="str">
-        <x:v>主語・述語が対応し、一文で意味が完結</x:v>
+        <x:v>誰のことか、何について書いたか、最後まで一文を読むと分かる</x:v>
       </x:c>
       <x:c r="F5" s="55" t="str">
-        <x:v>3問連続合格</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格</x:v>
       </x:c>
       <x:c r="G5" s="58" t="str">
         <x:v>個別設定可</x:v>
@@ -1029,13 +1029,13 @@
         <x:v>一文を正確にする</x:v>
       </x:c>
       <x:c r="D6" s="46" t="str">
-        <x:v>修飾・助詞・接続を整え、意味が明確な一文を書く</x:v>
+        <x:v>説明する言葉を近くに置き、「が・を・に・で」などを選んで、読みやすい一文を書く</x:v>
       </x:c>
       <x:c r="E6" s="46" t="str">
-        <x:v>修飾関係と助詞が適切で、意味が一義的</x:v>
+        <x:v>誰が何をする文なのか、読み手が迷わず一つの意味に読める</x:v>
       </x:c>
       <x:c r="F6" s="55" t="str">
-        <x:v>3問連続合格</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格</x:v>
       </x:c>
       <x:c r="G6" s="58" t="str">
         <x:v>個別設定可</x:v>
@@ -1052,13 +1052,13 @@
         <x:v>問いへの立場を示す</x:v>
       </x:c>
       <x:c r="D7" s="46" t="str">
-        <x:v>テーマへの主張を一文で明確に書く</x:v>
+        <x:v>問いに対する自分の答えを、一文だけで分かるように書く</x:v>
       </x:c>
       <x:c r="E7" s="46" t="str">
-        <x:v>問いに答え、自分の立場が明示</x:v>
+        <x:v>賛成・反対、または何を大切にする考えなのかが分かる</x:v>
       </x:c>
       <x:c r="F7" s="55" t="str">
-        <x:v>3問連続合格</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格</x:v>
       </x:c>
       <x:c r="G7" s="58" t="str">
         <x:v>個別設定可</x:v>
@@ -1075,13 +1075,13 @@
         <x:v>主張と理由を結ぶ</x:v>
       </x:c>
       <x:c r="D8" s="46" t="str">
-        <x:v>主張→理由の二文構成を書く</x:v>
+        <x:v>一文目に意見、二文目に「なぜそう考えるのか」を書く</x:v>
       </x:c>
       <x:c r="E8" s="46" t="str">
-        <x:v>因果関係が明確で、理由が主張の言い換えでない</x:v>
+        <x:v>二文目が一文目の言い換えではなく、意見を選んだ理由になっている</x:v>
       </x:c>
       <x:c r="F8" s="55" t="str">
-        <x:v>3問連続合格</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格</x:v>
       </x:c>
       <x:c r="G8" s="58" t="str">
         <x:v>個別設定可</x:v>
@@ -1098,13 +1098,13 @@
         <x:v>理由を具体化する</x:v>
       </x:c>
       <x:c r="D9" s="46" t="str">
-        <x:v>理由の中身を説明して説得力を高める</x:v>
+        <x:v>理由によって何が起こり、どのような結果になるのかまで書く</x:v>
       </x:c>
       <x:c r="E9" s="46" t="str">
-        <x:v>理由が抽象語の反復でなく、因果を説明</x:v>
+        <x:v>「よいから」「大切だから」で終わらず、起こることと結果が分かる</x:v>
       </x:c>
       <x:c r="F9" s="55" t="str">
-        <x:v>3問連続合格</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格</x:v>
       </x:c>
       <x:c r="G9" s="58" t="str">
         <x:v>個別設定可</x:v>
@@ -1121,13 +1121,13 @@
         <x:v>根拠を具体化する</x:v>
       </x:c>
       <x:c r="D10" s="46" t="str">
-        <x:v>主張→理由→具体例の三文構成を書く</x:v>
+        <x:v>一文目に意見、二文目に理由、三文目に理由が当てはまる具体例を書く</x:v>
       </x:c>
       <x:c r="E10" s="46" t="str">
-        <x:v>具体例が主張・理由に論理的に接続</x:v>
+        <x:v>具体例を読むと、理由が実際にどう当てはまるのか分かる</x:v>
       </x:c>
       <x:c r="F10" s="55" t="str">
-        <x:v>3問連続合格</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格</x:v>
       </x:c>
       <x:c r="G10" s="58" t="str">
         <x:v>個別設定可</x:v>
@@ -1144,13 +1144,13 @@
         <x:v>最小段落を作る</x:v>
       </x:c>
       <x:c r="D11" s="46" t="str">
-        <x:v>主張→理由→具体例→まとめの段落を書く</x:v>
+        <x:v>意見・理由・具体例・結論を一文ずつ書き、四文の段落を作る</x:v>
       </x:c>
       <x:c r="E11" s="46" t="str">
-        <x:v>まとめが主張と整合し、段落として完結</x:v>
+        <x:v>四文が同じ話題について書かれ、最後の文が最初の意見に戻っている</x:v>
       </x:c>
       <x:c r="F11" s="55" t="str">
-        <x:v>3問連続合格</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格</x:v>
       </x:c>
       <x:c r="G11" s="58" t="str">
         <x:v>個別設定可</x:v>
@@ -1167,13 +1167,13 @@
         <x:v>論旨を捉える</x:v>
       </x:c>
       <x:c r="D12" s="46" t="str">
-        <x:v>課題文の主張・理由・具体例・結論を区別する</x:v>
+        <x:v>課題文から、筆者の意見・理由・具体例・反対意見や例外を見つけて分ける</x:v>
       </x:c>
       <x:c r="E12" s="46" t="str">
-        <x:v>各要素を本文の根拠に基づいて抽出</x:v>
+        <x:v>分けた内容が課題文のどの言葉や文に基づくのか分かる</x:v>
       </x:c>
       <x:c r="F12" s="55" t="str">
-        <x:v>3問連続合格</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格</x:v>
       </x:c>
       <x:c r="G12" s="58" t="str">
         <x:v>個別設定可</x:v>
@@ -1190,13 +1190,13 @@
         <x:v>意見を混ぜずに要約する</x:v>
       </x:c>
       <x:c r="D13" s="46" t="str">
-        <x:v>課題文の論旨を過不足なく要約する</x:v>
+        <x:v>筆者が最も伝えたいことと重要な理由を残し、自分の意見を入れずに短くまとめる</x:v>
       </x:c>
       <x:c r="E13" s="46" t="str">
-        <x:v>筆者の主張と根拠を保ち、私見を混入させない</x:v>
+        <x:v>筆者の意見と理由が残り、「私は」などの自分の意見が入っていない</x:v>
       </x:c>
       <x:c r="F13" s="55" t="str">
-        <x:v>3問連続合格</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格</x:v>
       </x:c>
       <x:c r="G13" s="58" t="str">
         <x:v>個別設定可</x:v>
@@ -1213,13 +1213,13 @@
         <x:v>課題文を踏まえ意見を作る</x:v>
       </x:c>
       <x:c r="D14" s="46" t="str">
-        <x:v>要約→立場→理由を書き、論拠を示す</x:v>
+        <x:v>課題文の内容を一つ取り上げ、自分の意見と、その意見を選ぶ理由を書く</x:v>
       </x:c>
       <x:c r="E14" s="46" t="str">
-        <x:v>意見と課題文の関係が明確で、根拠がある</x:v>
+        <x:v>課題文のどの内容をもとに考えたかと、自分の意見・理由が分かる</x:v>
       </x:c>
       <x:c r="F14" s="55" t="str">
-        <x:v>3問連続合格</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格</x:v>
       </x:c>
       <x:c r="G14" s="58" t="str">
         <x:v>個別設定可</x:v>
@@ -1236,13 +1236,13 @@
         <x:v>多面的に考える</x:v>
       </x:c>
       <x:c r="D15" s="46" t="str">
-        <x:v>反対意見または別の立場を扱い、自説を検討する</x:v>
+        <x:v>反対の立場を正確に紹介し、納得できる点を認めたうえで、自分の意見を書く</x:v>
       </x:c>
       <x:c r="E15" s="46" t="str">
-        <x:v>別視点を公平に示し、自説との関係を説明</x:v>
+        <x:v>反対の立場を実際より弱くせず、それでも自分の意見を選ぶ理由が分かる</x:v>
       </x:c>
       <x:c r="F15" s="55" t="str">
-        <x:v>3問連続合格</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格</x:v>
       </x:c>
       <x:c r="G15" s="58" t="str">
         <x:v>個別設定可</x:v>
@@ -1259,13 +1259,13 @@
         <x:v>短い小論文を完成させる</x:v>
       </x:c>
       <x:c r="D16" s="46" t="str">
-        <x:v>指定字数内で構成を保った小論文を書く</x:v>
+        <x:v>最初に意見を示し、途中で理由と具体例を説明し、最後に結論を書く</x:v>
       </x:c>
       <x:c r="E16" s="46" t="str">
-        <x:v>主張・理由・具体例・結論が一貫</x:v>
+        <x:v>最初の意見、理由、具体例、最後の結論が同じ答えを支えている</x:v>
       </x:c>
       <x:c r="F16" s="55" t="str">
-        <x:v>3問連続合格</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格</x:v>
       </x:c>
       <x:c r="G16" s="58" t="str">
         <x:v>個別設定可</x:v>
@@ -1282,13 +1282,13 @@
         <x:v>本番形式で統合する</x:v>
       </x:c>
       <x:c r="D17" s="47" t="str">
-        <x:v>課題文を読み、時間内に小論文を書き切る</x:v>
+        <x:v>設問への答えを示し、理由・具体例・別の立場を扱い、最後に答えへ戻る</x:v>
       </x:c>
       <x:c r="E17" s="47" t="str">
-        <x:v>日本語文成立チェック、論理構成、一定水準を満たせば合格。合格後も改善コメントを返す</x:v>
+        <x:v>設問に答え、理由・具体例・別の立場・結論が途中でずれていない</x:v>
       </x:c>
       <x:c r="F17" s="56" t="str">
-        <x:v>基準到達後も、学習者が終了を選ぶまで継続</x:v>
+        <x:v>通常10問合格後、進級テストで累計3問合格して全課程修了</x:v>
       </x:c>
       <x:c r="G17" s="34" t="str">
         <x:v>管理者承認は不要。質が十分なら、次の課題へ進む選択肢を提案する</x:v>
@@ -1300,7 +1300,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4a74c6abdb141de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a25a1801efb4342"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1386,13 +1386,13 @@
         <x:v>主語・述語</x:v>
       </x:c>
       <x:c r="E4" s="45" t="str">
-        <x:v>主語と述語が対応している</x:v>
+        <x:v>「誰が・何が」と「どうする・どのようだ」が組み合わさっている</x:v>
       </x:c>
       <x:c r="F4" s="54" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G4" s="45" t="str">
-        <x:v>例: 『私は読書が好きだ。』のように、誰がどうであるかが読める</x:v>
+        <x:v>例：「私は読書が好きだ。」なら、「私は」と「好きだ」が対応している</x:v>
       </x:c>
       <x:c r="H4" s="57" t="str"/>
     </x:row>
@@ -1410,13 +1410,13 @@
         <x:v>文の完結</x:v>
       </x:c>
       <x:c r="E5" s="46" t="str">
-        <x:v>一文で意味が完結している</x:v>
+        <x:v>文の最後まで書かれ、一文だけで意味が分かる</x:v>
       </x:c>
       <x:c r="F5" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G5" s="46" t="str">
-        <x:v>文末まで書き、途中で終わらない</x:v>
+        <x:v>「。」などを付け、言いかけのまま終わらせない</x:v>
       </x:c>
       <x:c r="H5" s="58" t="str"/>
     </x:row>
@@ -1434,13 +1434,13 @@
         <x:v>修飾関係</x:v>
       </x:c>
       <x:c r="E6" s="46" t="str">
-        <x:v>修飾語が何を修飾するか明確である</x:v>
+        <x:v>説明する言葉が、説明される言葉の近くに置かれている</x:v>
       </x:c>
       <x:c r="F6" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G6" s="46" t="str">
-        <x:v>長い修飾語でも、対象語との関係を確認する</x:v>
+        <x:v>一つの説明が二つの言葉にかかるように読めないかを見る</x:v>
       </x:c>
       <x:c r="H6" s="58" t="str"/>
     </x:row>
@@ -1458,13 +1458,13 @@
         <x:v>助詞・接続</x:v>
       </x:c>
       <x:c r="E7" s="46" t="str">
-        <x:v>助詞と接続が意味に合っている</x:v>
+        <x:v>「が・を・に・で」などが、誰が何をするかに合っている</x:v>
       </x:c>
       <x:c r="F7" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G7" s="46" t="str">
-        <x:v>『ため』『ので』は因果関係がある場合だけ使う</x:v>
+        <x:v>使った言葉を入れ替えたときに意味が変わらないか、文全体で判断する</x:v>
       </x:c>
       <x:c r="H7" s="58" t="str"/>
     </x:row>
@@ -1482,13 +1482,13 @@
         <x:v>立場</x:v>
       </x:c>
       <x:c r="E8" s="46" t="str">
-        <x:v>テーマへの立場が明確に書かれている</x:v>
+        <x:v>問いに対する自分の答えが、一文だけで分かる</x:v>
       </x:c>
       <x:c r="F8" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G8" s="46" t="str">
-        <x:v>賛成・反対、または何を重視するかを一文で示す</x:v>
+        <x:v>賛成・反対、または何を大切にする考えなのかを示す</x:v>
       </x:c>
       <x:c r="H8" s="58" t="str"/>
     </x:row>
@@ -1506,13 +1506,13 @@
         <x:v>因果関係</x:v>
       </x:c>
       <x:c r="E9" s="46" t="str">
-        <x:v>理由が主張を支え、因果関係が明確である</x:v>
+        <x:v>二文目を読むと、一文目の意見を選んだ理由が分かる</x:v>
       </x:c>
       <x:c r="F9" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G9" s="46" t="str">
-        <x:v>理由が主張の言い換えだけにならない</x:v>
+        <x:v>二文目が一文目の言い換えだけになっていないかを見る</x:v>
       </x:c>
       <x:c r="H9" s="58" t="str"/>
     </x:row>
@@ -1530,13 +1530,13 @@
         <x:v>理由の具体性</x:v>
       </x:c>
       <x:c r="E10" s="46" t="str">
-        <x:v>理由の中身が説明されている</x:v>
+        <x:v>理由によって何が起こり、どのような結果になるのかが書かれている</x:v>
       </x:c>
       <x:c r="F10" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G10" s="46" t="str">
-        <x:v>抽象語を具体的な因果へ分解する</x:v>
+        <x:v>「便利だから」などで止めず、誰に何が起こるのかまで読む</x:v>
       </x:c>
       <x:c r="H10" s="58" t="str"/>
     </x:row>
@@ -1554,13 +1554,13 @@
         <x:v>具体例の関連</x:v>
       </x:c>
       <x:c r="E11" s="46" t="str">
-        <x:v>具体例が主張・理由を支えている</x:v>
+        <x:v>具体例が、直前の理由が実際に当てはまる場面になっている</x:v>
       </x:c>
       <x:c r="F11" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G11" s="46" t="str">
-        <x:v>例だけを増やさず、何を示す例かを明確にする</x:v>
+        <x:v>例を読んだときに、なぜ意見に納得できるのか分かるかを見る</x:v>
       </x:c>
       <x:c r="H11" s="58" t="str"/>
     </x:row>
@@ -1578,13 +1578,13 @@
         <x:v>まとめ</x:v>
       </x:c>
       <x:c r="E12" s="46" t="str">
-        <x:v>まとめが主張と整合し、段落が完結している</x:v>
+        <x:v>四文が同じ話題について書かれ、最後の文が最初の意見に戻っている</x:v>
       </x:c>
       <x:c r="F12" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G12" s="46" t="str">
-        <x:v>新しい論点を最後に追加しない</x:v>
+        <x:v>最後の文で新しい話を始めていないかを見る</x:v>
       </x:c>
       <x:c r="H12" s="58" t="str"/>
     </x:row>
@@ -1602,13 +1602,13 @@
         <x:v>根拠抽出</x:v>
       </x:c>
       <x:c r="E13" s="46" t="str">
-        <x:v>課題文中の根拠に基づき構造を捉える</x:v>
+        <x:v>分けた内容が、課題文のどの言葉や文に基づくのか分かる</x:v>
       </x:c>
       <x:c r="F13" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G13" s="46" t="str">
-        <x:v>推測だけで要素を決めない</x:v>
+        <x:v>学習者の推測だけで、筆者の意見や理由を決めない</x:v>
       </x:c>
       <x:c r="H13" s="58" t="str"/>
     </x:row>
@@ -1626,13 +1626,13 @@
         <x:v>私見の分離</x:v>
       </x:c>
       <x:c r="E14" s="46" t="str">
-        <x:v>筆者の意見と自分の意見を混同しない</x:v>
+        <x:v>筆者の意見と理由を残し、自分の意見を加えていない</x:v>
       </x:c>
       <x:c r="F14" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G14" s="46" t="str">
-        <x:v>『私は』を入れない</x:v>
+        <x:v>「私は」など、筆者にはない意見を入れない</x:v>
       </x:c>
       <x:c r="H14" s="58" t="str"/>
     </x:row>
@@ -1650,13 +1650,13 @@
         <x:v>論拠</x:v>
       </x:c>
       <x:c r="E15" s="46" t="str">
-        <x:v>自分の立場を支える理由が示されている</x:v>
+        <x:v>課題文のどの内容をもとに考えたかと、自分の意見・理由が分かる</x:v>
       </x:c>
       <x:c r="F15" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G15" s="46" t="str">
-        <x:v>課題文の内容との接点を示す</x:v>
+        <x:v>課題文と関係のない理由だけで意見を書かない</x:v>
       </x:c>
       <x:c r="H15" s="58" t="str"/>
     </x:row>
@@ -1674,13 +1674,13 @@
         <x:v>別視点</x:v>
       </x:c>
       <x:c r="E16" s="46" t="str">
-        <x:v>反対意見等を正確に示し、自説との関係を説明する</x:v>
+        <x:v>反対の立場を正確に示し、それでも自分の意見を選ぶ理由を書いている</x:v>
       </x:c>
       <x:c r="F16" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G16" s="46" t="str">
-        <x:v>相手の意見をわざと弱くしない</x:v>
+        <x:v>相手の意見を実際より弱く言い換えない</x:v>
       </x:c>
       <x:c r="H16" s="58" t="str"/>
     </x:row>
@@ -1698,13 +1698,13 @@
         <x:v>一貫性</x:v>
       </x:c>
       <x:c r="E17" s="46" t="str">
-        <x:v>主張・理由・具体例・結論が矛盾しない</x:v>
+        <x:v>最初の意見、理由、具体例、最後の結論が同じ答えを支えている</x:v>
       </x:c>
       <x:c r="F17" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G17" s="46" t="str">
-        <x:v>各段落が中心主張を支える</x:v>
+        <x:v>途中で別の答えへ変わっていないか、段落ごとに読む</x:v>
       </x:c>
       <x:c r="H17" s="58" t="str"/>
     </x:row>
@@ -1722,13 +1722,13 @@
         <x:v>合格判定</x:v>
       </x:c>
       <x:c r="E18" s="47" t="str">
-        <x:v>日本語文成立チェックがcleanであり、設問に適合し、主張・根拠・論理展開が一貫し、小論文として一定水準に到達している</x:v>
+        <x:v>設問に答え、読み手が意味を迷わず読め、理由・具体例・結論が同じ答えを支えている</x:v>
       </x:c>
       <x:c r="F18" s="56" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G18" s="47" t="str">
-        <x:v>管理者の承認ではなく、定義済みの到達基準でAIが判定する。改善点が残っていても、基準を満たせば合格にする</x:v>
+        <x:v>改善できる点が残っていても、この条件を満たせば合格にする</x:v>
       </x:c>
       <x:c r="H18" s="34" t="str">
         <x:v>合格後の改善コメントを合否理由と混同しない</x:v>
@@ -1748,13 +1748,13 @@
         <x:v>日本語文成立</x:v>
       </x:c>
       <x:c r="E19" s="45" t="str">
-        <x:v>全提出文に構造上の問題がない（status: clean）</x:v>
-      </x:c>
-      <x:c r="F19" s="86" t="str">
+        <x:v>誰が何をする文なのかが分かり、言葉の位置やつなぎ方で意味が崩れていない</x:v>
+      </x:c>
+      <x:c r="F19" s="54" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G19" s="45" t="str">
-        <x:v>ねじれ文、助詞・修飾・接続・因果関係の破綻を先に確認する</x:v>
+        <x:v>文を一つずつ読み、どの言葉の組み合わせで迷うのかを特定する</x:v>
       </x:c>
       <x:c r="H19" s="88" t="str"/>
     </x:row>
@@ -1772,13 +1772,13 @@
         <x:v>論旨の一貫性</x:v>
       </x:c>
       <x:c r="E20" s="46" t="str">
-        <x:v>主張、根拠、具体例、結論の関係が一貫し、設問に答えている</x:v>
-      </x:c>
-      <x:c r="F20" s="87" t="str">
+        <x:v>意見、理由、具体例、結論が途中でずれず、設問への答えになっている</x:v>
+      </x:c>
+      <x:c r="F20" s="55" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="G20" s="46" t="str">
-        <x:v>段落ごとの役割と、結論が主張に対応するかを確認する</x:v>
+        <x:v>各段落が何を説明し、最後の結論が最初の答えに戻るかを見る</x:v>
       </x:c>
       <x:c r="H20" s="89" t="str"/>
     </x:row>
@@ -1796,13 +1796,13 @@
         <x:v>改善コメント</x:v>
       </x:c>
       <x:c r="E21" s="46" t="str">
-        <x:v>合格後も、より明確にできる点・根拠を深められる点をコメントとして残す</x:v>
-      </x:c>
-      <x:c r="F21" s="87" t="str">
+        <x:v>合格後も、さらに分かりやすくできる箇所や、理由を詳しくできる箇所を具体的に伝える</x:v>
+      </x:c>
+      <x:c r="F21" s="55" t="str">
         <x:v>合格後も実施</x:v>
       </x:c>
       <x:c r="G21" s="46" t="str">
-        <x:v>改善点は不合格理由ではない。再提出時は前回の改善点への対応を添削し、新たな改善点も返す</x:v>
+        <x:v>改善案は不合格理由と分け、どの語句をどう変えるかを書く</x:v>
       </x:c>
       <x:c r="H21" s="89" t="str">
         <x:v>学習者が終了を選ぶまで繰り返す</x:v>
@@ -1821,14 +1821,14 @@
       <x:c r="D22" t="str">
         <x:v>次課題の提案</x:v>
       </x:c>
-      <x:c r="E22" t="str">
-        <x:v>日本語・論理構成・小論文としての到達水準が十分で、次の課題へ進むことが学習上有効と判断できる</x:v>
-      </x:c>
-      <x:c r="F22" t="str">
+      <x:c r="E22" s="104" t="str">
+        <x:v>今の文章で十分に学べた場合は、次の課題へ進む選択肢と、その理由を伝える</x:v>
+      </x:c>
+      <x:c r="F22" s="104" t="str">
         <x:v>条件付きで実施</x:v>
       </x:c>
-      <x:c r="G22" t="str">
-        <x:v>合格後も改善点は返す。そのうえで、現論文を終了して次の課題へ進む選択肢を、理由を添えて穏やかに提案する。強制しない</x:v>
+      <x:c r="G22" s="104" t="str">
+        <x:v>続けて直すか次へ進むかは学習者が選べるようにする</x:v>
       </x:c>
       <x:c r="H22" t="str">
         <x:v>学習者は継続添削か次課題への移行かを選べる</x:v>
@@ -1847,14 +1847,14 @@
       <x:c r="D23" t="str">
         <x:v>論旨の一貫性</x:v>
       </x:c>
-      <x:c r="E23" t="str">
-        <x:v>主張、根拠、具体例、結論の関係が一貫し、設問に答えている</x:v>
-      </x:c>
-      <x:c r="F23" t="str">
-        <x:v>必須</x:v>
-      </x:c>
-      <x:c r="G23" t="str">
-        <x:v>段落ごとの役割と、結論が主張に対応するかを確認する</x:v>
+      <x:c r="E23" s="104" t="str">
+        <x:v>意見、理由、具体例、結論が途中でずれず、設問への答えになっている</x:v>
+      </x:c>
+      <x:c r="F23" s="104" t="str">
+        <x:v>必須</x:v>
+      </x:c>
+      <x:c r="G23" s="104" t="str">
+        <x:v>各段落が何を説明し、最後の結論が最初の答えに戻るかを見る</x:v>
       </x:c>
       <x:c r="H23" t="str"/>
     </x:row>
@@ -1871,14 +1871,14 @@
       <x:c r="D24" t="str">
         <x:v>改善コメント</x:v>
       </x:c>
-      <x:c r="E24" t="str">
-        <x:v>合格後も、より明確にできる点・根拠を深められる点をコメントとして残す</x:v>
-      </x:c>
-      <x:c r="F24" t="str">
+      <x:c r="E24" s="104" t="str">
+        <x:v>合格後も、さらに分かりやすくできる箇所や、理由を詳しくできる箇所を具体的に伝える</x:v>
+      </x:c>
+      <x:c r="F24" s="104" t="str">
         <x:v>合格後も実施</x:v>
       </x:c>
-      <x:c r="G24" t="str">
-        <x:v>改善点は不合格理由ではない。再提出時は前回の改善点への対応を添削し、新たな改善点も返す</x:v>
+      <x:c r="G24" s="104" t="str">
+        <x:v>改善案は不合格理由と分け、どの語句をどう変えるかを書く</x:v>
       </x:c>
       <x:c r="H24" t="str">
         <x:v>学習者が終了を選ぶまで繰り返す</x:v>
@@ -1897,14 +1897,14 @@
       <x:c r="D25" t="str">
         <x:v>次課題の提案</x:v>
       </x:c>
-      <x:c r="E25" t="str">
-        <x:v>日本語・論理構成・小論文としての到達水準が十分で、次の課題へ進むことが学習上有効と判断できる</x:v>
-      </x:c>
-      <x:c r="F25" t="str">
+      <x:c r="E25" s="104" t="str">
+        <x:v>今の文章で十分に学べた場合は、次の課題へ進む選択肢と、その理由を伝える</x:v>
+      </x:c>
+      <x:c r="F25" s="104" t="str">
         <x:v>条件付きで実施</x:v>
       </x:c>
-      <x:c r="G25" t="str">
-        <x:v>合格後も改善点は返す。そのうえで、現論文を終了して次の課題へ進む選択肢を、理由を添えて穏やかに提案する。強制しない</x:v>
+      <x:c r="G25" s="104" t="str">
+        <x:v>続けて直すか次へ進むかは学習者が選べるようにする</x:v>
       </x:c>
       <x:c r="H25" t="str">
         <x:v>学習者は継続添削か次課題への移行かを選べる</x:v>
@@ -1916,7 +1916,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4b83240f45347e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45750650bfb64782"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1974,7 +1974,7 @@
         <x:v>管理者メモ</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="4" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A4" s="59" t="str">
         <x:v>subject_predicate</x:v>
       </x:c>
@@ -1982,17 +1982,17 @@
         <x:v>主語・述語</x:v>
       </x:c>
       <x:c r="C4" s="45" t="str">
-        <x:v>誰が／何が と、どうする／どうである の対応が取れているか</x:v>
+        <x:v>「誰が・何が」に当たる言葉と、「どうする・どのようだ」に当たる言葉が組み合わさっているか</x:v>
       </x:c>
       <x:c r="D4" s="45" t="str">
         <x:v>主語と述語が対応しない、述語が欠ける</x:v>
       </x:c>
       <x:c r="E4" s="45" t="str">
-        <x:v>どの語とどの語の対応が崩れているかを説明する</x:v>
+        <x:v>答案中の二つの言葉を示し、誰について何を述べる文に直すのかを書く</x:v>
       </x:c>
       <x:c r="F4" s="57" t="str"/>
     </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
+    <x:row r="5" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A5" s="60" t="str">
         <x:v>modifier</x:v>
       </x:c>
@@ -2000,17 +2000,17 @@
         <x:v>修飾関係</x:v>
       </x:c>
       <x:c r="C5" s="46" t="str">
-        <x:v>修飾語が何を修飾するか一義的か</x:v>
+        <x:v>説明する言葉が、説明される言葉の近くにあり、別の意味に読まれないか</x:v>
       </x:c>
       <x:c r="D5" s="46" t="str">
         <x:v>別の語に係るように読める、係り先がない</x:v>
       </x:c>
       <x:c r="E5" s="46" t="str">
-        <x:v>読者がどのように読み違えるかを示す</x:v>
+        <x:v>読み手が迷う二つの読み方を示し、説明する言葉をどの言葉の前へ移すかを書く</x:v>
       </x:c>
       <x:c r="F5" s="58" t="str"/>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+    <x:row r="6" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A6" s="60" t="str">
         <x:v>particle</x:v>
       </x:c>
@@ -2018,17 +2018,17 @@
         <x:v>助詞</x:v>
       </x:c>
       <x:c r="C6" s="46" t="str">
-        <x:v>助詞が語句の関係を正しく示しているか</x:v>
+        <x:v>「が・を・に・で」などによって、誰が何をするのかが正しく読めるか</x:v>
       </x:c>
       <x:c r="D6" s="46" t="str">
         <x:v>助詞の欠落・誤用で役割が分からない</x:v>
       </x:c>
       <x:c r="E6" s="46" t="str">
-        <x:v>何と何の関係を示す助詞かを説明する</x:v>
+        <x:v>使われている言葉を示し、何へ置き換えると誰が何をする文になるのかを書く</x:v>
       </x:c>
       <x:c r="F6" s="58" t="str"/>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+    <x:row r="7" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A7" s="60" t="str">
         <x:v>connection</x:v>
       </x:c>
@@ -2036,17 +2036,17 @@
         <x:v>接続</x:v>
       </x:c>
       <x:c r="C7" s="46" t="str">
-        <x:v>接続語・接続助詞が前後の関係に合うか</x:v>
+        <x:v>「しかし」「そのため」などが、前後の内容の関係に合っているか</x:v>
       </x:c>
       <x:c r="D7" s="46" t="str">
         <x:v>対比・因果・追加の関係が不一致</x:v>
       </x:c>
       <x:c r="E7" s="46" t="str">
-        <x:v>接続語が本来示す関係と実際の関係を説明する</x:v>
+        <x:v>前後が反対・理由と結果・付け足しのどれなのかを示し、合うつなぎ言葉を書く</x:v>
       </x:c>
       <x:c r="F7" s="58" t="str"/>
     </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
+    <x:row r="8" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A8" s="60" t="str">
         <x:v>parallelism</x:v>
       </x:c>
@@ -2054,17 +2054,17 @@
         <x:v>並列</x:v>
       </x:c>
       <x:c r="C8" s="46" t="str">
-        <x:v>並べた語句・述語の形や対象がそろうか</x:v>
+        <x:v>並べた言葉や動作が、同じ種類・同じ形になっているか</x:v>
       </x:c>
       <x:c r="D8" s="46" t="str">
         <x:v>形・対象・時制が不揃いで関係が不明</x:v>
       </x:c>
       <x:c r="E8" s="46" t="str">
-        <x:v>何を並列にしたい文かを明示する</x:v>
+        <x:v>何と何を並べたい文なのかを示し、語尾や形をそろえた書き方を示す</x:v>
       </x:c>
       <x:c r="F8" s="58" t="str"/>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+    <x:row r="9" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A9" s="60" t="str">
         <x:v>omission</x:v>
       </x:c>
@@ -2072,17 +2072,17 @@
         <x:v>省略</x:v>
       </x:c>
       <x:c r="C9" s="46" t="str">
-        <x:v>省略された主語・目的語が文脈から復元できるか</x:v>
+        <x:v>省かれた「誰が・何を」が、前後を読めば一つに決まるか</x:v>
       </x:c>
       <x:c r="D9" s="46" t="str">
         <x:v>誰が／何を が特定できない</x:v>
       </x:c>
       <x:c r="E9" s="46" t="str">
-        <x:v>補うべき情報を質問形式で示す</x:v>
+        <x:v>分からない情報を「誰が〜するのですか」のような質問で示す</x:v>
       </x:c>
       <x:c r="F9" s="58" t="str"/>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+    <x:row r="10" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A10" s="60" t="str">
         <x:v>reference</x:v>
       </x:c>
@@ -2090,17 +2090,17 @@
         <x:v>指示語</x:v>
       </x:c>
       <x:c r="C10" s="46" t="str">
-        <x:v>指示語が何を指すか明確か</x:v>
+        <x:v>「これ・それ・このこと」が、どの言葉や文を指すか一つに決まるか</x:v>
       </x:c>
       <x:c r="D10" s="46" t="str">
         <x:v>これ・それ等の参照先が複数または不明</x:v>
       </x:c>
       <x:c r="E10" s="46" t="str">
-        <x:v>指示語の参照先を具体的に書くよう促す</x:v>
+        <x:v>指している内容を具体的な言葉に置き換えるよう伝える</x:v>
       </x:c>
       <x:c r="F10" s="58" t="str"/>
     </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
+    <x:row r="11" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A11" s="60" t="str">
         <x:v>tense</x:v>
       </x:c>
@@ -2108,17 +2108,17 @@
         <x:v>時制</x:v>
       </x:c>
       <x:c r="C11" s="46" t="str">
-        <x:v>時制の移り変わりが意味に合うか</x:v>
+        <x:v>過去・現在・未来の書き方が、出来事の順番に合っているか</x:v>
       </x:c>
       <x:c r="D11" s="46" t="str">
         <x:v>過去・現在・未来の関係が不自然</x:v>
       </x:c>
       <x:c r="E11" s="46" t="str">
-        <x:v>いつの出来事かを統一するよう促す</x:v>
+        <x:v>いつ起きたことかを示し、どの語尾を過去・現在・未来に直すかを書く</x:v>
       </x:c>
       <x:c r="F11" s="58" t="str"/>
     </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
+    <x:row r="12" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A12" s="60" t="str">
         <x:v>logical_relation</x:v>
       </x:c>
@@ -2126,17 +2126,17 @@
         <x:v>論理関係</x:v>
       </x:c>
       <x:c r="C12" s="46" t="str">
-        <x:v>一文内・文間の因果や対比が成立するか</x:v>
+        <x:v>理由から結果へ、または前の文から後の文へ、内容が飛ばずにつながっているか</x:v>
       </x:c>
       <x:c r="D12" s="46" t="str">
         <x:v>原因と結果、前提と結論の関係がつながらない</x:v>
       </x:c>
       <x:c r="E12" s="46" t="str">
-        <x:v>前件から後件へ何が起きるかを補うよう促す</x:v>
+        <x:v>間に足りない出来事や説明を示し、どこに加えるかを書く</x:v>
       </x:c>
       <x:c r="F12" s="58" t="str"/>
     </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
+    <x:row r="13" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A13" s="61" t="str">
         <x:v>typo</x:v>
       </x:c>
@@ -2144,13 +2144,13 @@
         <x:v>誤字・脱字</x:v>
       </x:c>
       <x:c r="C13" s="47" t="str">
-        <x:v>表記の誤りが意味理解を妨げるか</x:v>
+        <x:v>書き間違いや抜けた文字によって、意味が変わったり読めなくなったりしていないか</x:v>
       </x:c>
       <x:c r="D13" s="47" t="str">
         <x:v>誤字・脱字により別の意味になる</x:v>
       </x:c>
       <x:c r="E13" s="47" t="str">
-        <x:v>表記を示し、文構造の問題とは区別する</x:v>
+        <x:v>該当する言葉と正しい表記を示し、文章の組み立ての問題とは分けて伝える</x:v>
       </x:c>
       <x:c r="F13" s="34" t="str"/>
     </x:row>
@@ -2160,7 +2160,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc8a29fd8b914214"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68bea3f94b26415c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2232,7 +2232,7 @@
         <x:v>学習者に不要なコメントを出さない。</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+    <x:row r="6" ht="54" hidden="0" customHeight="1">
       <x:c r="A6" s="64" t="str">
         <x:v>共通</x:v>
       </x:c>
@@ -2240,10 +2240,10 @@
         <x:v>根拠</x:v>
       </x:c>
       <x:c r="C6" s="65" t="str">
-        <x:v>『不自然』だけで終えず、語句間の関係を説明する</x:v>
+        <x:v>「不自然」「助詞を確認」「関係を明確に」だけで終えず、答案中の語句を示し、どの言葉をどこへ移す・何へ置き換える・何の後に加えるかを説明する</x:v>
       </x:c>
       <x:c r="D6" s="58" t="str">
-        <x:v>diagnosis と reader_interpretation を必須にする。</x:v>
+        <x:v>学習者が次の提出で実行できるコメントにする。専門用語を使う場合は、同じ文で意味や例を添える。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2282,10 +2282,10 @@
         <x:v>進級</x:v>
       </x:c>
       <x:c r="C9" s="65" t="str">
-        <x:v>3問連続合格を標準とする</x:v>
+        <x:v>通常トレーニング10問合格後、進級テストで累計3問合格を標準とする</x:v>
       </x:c>
       <x:c r="D9" s="58" t="str">
-        <x:v>管理者が個別に変更できる。</x:v>
+        <x:v>必要合格数は学習者が1〜10問で変更できる。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -2302,102 +2302,116 @@
         <x:v>日本語構造を先に直す。</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="11" ht="33" hidden="0" customHeight="1">
       <x:c r="A11" s="90" t="str">
         <x:v>本番小論文</x:v>
       </x:c>
       <x:c r="B11" s="91" t="str">
         <x:v>合格</x:v>
       </x:c>
-      <x:c r="C11" s="91" t="str">
+      <x:c r="C11" s="63" t="str">
         <x:v>合格は『改善点がゼロ』ではなく、定義済みの到達基準を満たすこと</x:v>
       </x:c>
-      <x:c r="D11" s="88" t="str">
+      <x:c r="D11" s="84" t="str">
         <x:v>無限に改善可能な小論文でも、利用者が到達を実感できるようにする。</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="12" ht="39" hidden="0" customHeight="1">
       <x:c r="A12" s="92" t="str">
         <x:v>本番小論文</x:v>
       </x:c>
       <x:c r="B12" s="93" t="str">
         <x:v>合格後</x:v>
       </x:c>
-      <x:c r="C12" s="93" t="str">
+      <x:c r="C12" s="65" t="str">
         <x:v>合格後も改善点を具体的にコメントする。再提出時は前回コメントへの対応を確認し、新しい改善点を返す</x:v>
       </x:c>
-      <x:c r="D12" s="89" t="str">
+      <x:c r="D12" s="85" t="str">
         <x:v>合格・改善コメント・再提出添削を併存させる。</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
+    <x:row r="13" ht="28.5" hidden="0" customHeight="1">
       <x:c r="A13" s="92" t="str">
         <x:v>本番小論文</x:v>
       </x:c>
       <x:c r="B13" s="93" t="str">
         <x:v>終了</x:v>
       </x:c>
-      <x:c r="C13" s="93" t="str">
+      <x:c r="C13" s="65" t="str">
         <x:v>終了判定は学習者が『この論文を終了する』と選んだ時だけ行う</x:v>
       </x:c>
-      <x:c r="D13" s="89" t="str">
+      <x:c r="D13" s="85" t="str">
         <x:v>AIや管理者が改善余地を理由に学習を終わらせない。</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
+    <x:row r="14" ht="48" hidden="0" customHeight="1">
       <x:c r="A14" t="str">
         <x:v>本番小論文</x:v>
       </x:c>
       <x:c r="B14" t="str">
         <x:v>次課題の提案</x:v>
       </x:c>
-      <x:c r="C14" t="str">
+      <x:c r="C14" s="104" t="str">
         <x:v>次の課題へ進んでよい質に達した場合は、改善コメントとは別に『この論文を終了して次の課題へ進む』選択肢を理由付きで提案する。提案は強制しない</x:v>
       </x:c>
-      <x:c r="D14" t="str">
+      <x:c r="D14" s="104" t="str">
         <x:v>終わりのない改善に陥らず、学習者が納得して次へ進めるようにする。</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="39" customHeight="1">
       <x:c r="A15" t="str">
         <x:v>本番小論文</x:v>
       </x:c>
       <x:c r="B15" t="str">
         <x:v>合格後</x:v>
       </x:c>
-      <x:c r="C15" t="str">
+      <x:c r="C15" s="104" t="str">
         <x:v>合格後も改善点を具体的にコメントする。再提出時は前回コメントへの対応を確認し、新しい改善点を返す</x:v>
       </x:c>
-      <x:c r="D15" t="str">
+      <x:c r="D15" s="104" t="str">
         <x:v>合格・改善コメント・再提出添削を併存させる。</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="28.5" customHeight="1">
       <x:c r="A16" t="str">
         <x:v>本番小論文</x:v>
       </x:c>
       <x:c r="B16" t="str">
         <x:v>終了</x:v>
       </x:c>
-      <x:c r="C16" t="str">
+      <x:c r="C16" s="104" t="str">
         <x:v>終了判定は学習者が『この論文を終了する』と選んだ時だけ行う</x:v>
       </x:c>
-      <x:c r="D16" t="str">
+      <x:c r="D16" s="104" t="str">
         <x:v>AIや管理者が改善余地を理由に学習を終わらせない。</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" t="str">
         <x:v>本番小論文</x:v>
       </x:c>
       <x:c r="B17" t="str">
         <x:v>次課題の提案</x:v>
       </x:c>
-      <x:c r="C17" t="str">
+      <x:c r="C17" s="104" t="str">
         <x:v>次の課題へ進んでよい質に達した場合は、改善コメントとは別に『この論文を終了して次の課題へ進む』選択肢を理由付きで提案する。提案は強制しない</x:v>
       </x:c>
-      <x:c r="D17" t="str">
+      <x:c r="D17" s="104" t="str">
         <x:v>終わりのない改善に陥らず、学習者が納得して次へ進めるようにする。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="48" customHeight="1">
+      <x:c r="A18" s="104" t="str">
+        <x:v>問題提示</x:v>
+      </x:c>
+      <x:c r="B18" s="104" t="str">
+        <x:v>ヒント</x:v>
+      </x:c>
+      <x:c r="C18" s="104" t="str">
+        <x:v>原則二文程度とし、最初に着目する文章要素や書く順序を示し、次に読み手へどう伝わればよいかを示す。段階2は指定された基準文をそのまま使う</x:v>
+      </x:c>
+      <x:c r="D18" s="104" t="str">
+        <x:v>専門用語には具体例を添え、ローカル派生問題でも説明文を機械的に追加しない。全13段階で同じ文章レベルを保つ。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2406,7 +2420,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdc6aafa97974930"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd846a71b41ad4110"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>